<commit_message>
Rename section labels across role-expectations documents
</commit_message>
<xml_diff>
--- a/role-expectations/期待職能_福田会計.xlsx
+++ b/role-expectations/期待職能_福田会計.xlsx
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>職能</t>
+          <t>職階</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -622,29 +622,29 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>主な役割</t>
+          <t>テーマ</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>昇進試験＆条件</t>
+          <t>昇格の条件</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>期待職能</t>
+          <t>期待される役割</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>期待されるパフォーマンス
-（フロントオフィス）</t>
+          <t>測定指標1
+（関与先担当）</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>期待されるパフォーマンス
-（バックオフィス）</t>
+          <t>測定指標2
+（総務・経理）</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>ラーニングラダー必須書籍リスト</t>
+          <t>必要なインプット</t>
         </is>
       </c>
     </row>
@@ -1204,63 +1204,71 @@
     <row r="12" ht="14" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>※1.所内ハンドブック試験は半年に1回は受験（再受験）すること。</t>
+          <t>※0.測定指標1は関与先を担当する職員（フロントオフィス）、測定指標2は総務・経理（バックオフィス）に適用する。兼任者は両方を見る。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="14" customHeight="1">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>※2.宣言書：自身が期待職能、パフォーマンスを満たしていることを根拠と共に記した文書。</t>
+          <t>※1.所内ハンドブック試験は半年に1回は受験（再受験）すること。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>※3.読書は、レポートの提出に伴い、レポート1通ごとに2,000円の補助を支給します。</t>
+          <t>※2.宣言書：自身が期待職能、パフォーマンスを満たしていることを根拠と共に記した文書。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="14" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>※4.半年間の粗利と自分の給与を比較して、労働分配率を計算。新卒の給与は12ヶ月、中途採用の給与は6ヶ月分は労働分配率の計算上考慮しない。</t>
+          <t>※3.読書は、レポートの提出に伴い、レポート1通ごとに2,000円の補助を支給します。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="14" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>※5.期待売上高＝基本給上限×2×1.3×1.15×14（千円未満切上）。「グレード制度 基本給テーブル」と一致。</t>
+          <t>※4.半年間の粗利と自分の給与を比較して、労働分配率を計算。新卒の給与は12ヶ月、中途採用の給与は6ヶ月分は労働分配率の計算上考慮しない。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>※6.月平均残業30時間超の場合、評価グレードを引き下げる（S：2グレードダウン／SS〜SM：1グレードダウン／T1：考慮しない）。</t>
+          <t>※5.期待売上高＝基本給上限×2×1.3×1.15×14（千円未満切上）。「グレード制度 基本給テーブル」と一致。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>※7.タイトルが上がれば上がるほど、抽象度が高まりよく分からないことも多くなります。逆に言うと「意味が分かる人しか、その役職にはなれない」とも言えますね。</t>
+          <t>※6.月平均残業30時間超の場合、評価グレードを引き下げる（S：2グレードダウン／SS〜SM：1グレードダウン／T1：考慮しない）。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="14" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
+          <t>※7.タイトルが上がれば上がるほど、抽象度が高まりよく分からないことも多くなります。逆に言うと「意味が分かる人しか、その役職にはなれない」とも言えますね。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="14" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
           <t>※8.評価面談では、この表の文言そのものを使ってフィードバックする。文言は直属上司が起案し、代表が承認、上司から本人へ通知する。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A12:K12"/>
     <mergeCell ref="A18:K18"/>
+    <mergeCell ref="A20:K20"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A19:K19"/>

</xml_diff>

<commit_message>
Split M/SM and D/SD into separate levels with per-grade themes
</commit_message>
<xml_diff>
--- a/role-expectations/期待職能_福田会計.xlsx
+++ b/role-expectations/期待職能_福田会計.xlsx
@@ -69,7 +69,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -93,12 +93,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="003C69B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="008EA9DB"/>
+        <fgColor rgb="007B96D4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009DB3E0"/>
       </patternFill>
     </fill>
     <fill>
@@ -148,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -177,10 +187,10 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -205,6 +215,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -575,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -584,17 +606,17 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>期待職能　税理士法人福田会計（2026-08-13版）</t>
+          <t>期待職能　税理士法人福田会計（2026-08-15版）</t>
         </is>
       </c>
     </row>
@@ -658,7 +680,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="67.5" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>EP</t>
@@ -666,9 +688,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>執行社員
-－エグゼクティブ
-　パートナー</t>
+          <t>執行社員</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -688,11 +708,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>＜EPへの昇格要件＞
-所内ハンドブック試験（マネージャー用）
-半年間に10冊以上の読書（要レポート）
-宣言書＆面接試験
-税理士登録済であること</t>
+          <t>昇格先なし。EP1→EP3 のグレード内昇給のみ</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -704,9 +720,9 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>(1)労働分配率43%（部下の売上10%＆メンバーの売上5%計上※4）
-(2)15名以上の組織を運営できる
-(3)年商3,000万円規模の新サービス・新拠点を立ち上げた経験がある
+          <t>(1)労働分配率43%（部下の売上10%＆メンバーの売上5%計上）
+(2)15名以上の組織を運営できる【仮】
+(3)年商3,000万円規模の新サービス・新拠点を立ち上げた経験がある【仮】
 (4)期待売上高（3,516万円以上）を達成している</t>
         </is>
       </c>
@@ -725,7 +741,6 @@
       <c r="K3" s="5" t="inlineStr">
         <is>
           <t>ビジョナリー・カンパニー②
-アメーバ経営（稲盛和夫）
 人を動かす</t>
         </is>
       </c>
@@ -758,113 +773,180 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
+          <t>＜EPへの昇格要件＞
+所内ハンドブック試験（マネージャー用）【要決定】
+半年間に10冊以上の読書（要レポート）
+宣言書＆面接試験
+税理士登録済であること【仮】</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>＜有能な経営者＞
+(1)自分が経験のない分野でも、事業計画やプロジェクトプランを策定することができる人
+(2)法人目標の達成に向けて、自ら成長と貢献の機会を作り出し、目に見える成果をあげる人</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>(1)労働分配率43%（部下の売上10%＆メンバーの売上5%計上）
+(2)10名以上の組織を運営できる【仮】
+(3)代表から経営者代理としての信頼を得ている
+(4)数年後のビジョンを明確にして、組織によい刺激を与えている
+(5)ゼロから年商1,000万円以上のサービス・部門を立ち上げた経験がある【仮】</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>(1)投資判断や意思決定において、法人全体最適を見据えつつ、自掌握組織に有益な意思決定ができる</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>(1)財務コーチングの実技指導を行える
+(2)所内ハンドブックの更新を提案し、実際に更新ができる</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>経営者の条件（ドラッカー）
+アメーバ経営（稲盛和夫）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="67.5" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>拠点長</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>SD1〜SD3</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>2,763〜3,014万円</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>計画策定と事業推進</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
           <t>＜Pへの昇格要件＞
-所内ハンドブック試験（マネージャー用）
+所内ハンドブック試験（マネージャー用）【要決定】
 半年間に8冊以上の読書（要レポート）
 宣言書＆面接試験
-税理士登録済であること</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>＜有能な経営者＞
-(1)自分が経験のない分野でも事業計画やプロジェクトプランを策定することができる人
-(2)法人目標の達成に向けて、自ら成長と貢献の機会を作り出し、目に見える成果をあげる人</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>(1)労働分配率43%（部下の売上10%＆メンバーの売上5%計上※4）
-(2)10名以上の組織を運営できる
-(3)代表から経営者代理としての信頼を得ている
-(4)数年後のビジョンを明確にして、組織によい刺激を与える
-(5)ゼロから年商1,000万円以上のサービス・部門を立ち上げた経験がある</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>(1)投資判断や意思決定において、法人全体最適を見据えつつ、自掌握組織に有益な意思決定ができる</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>(1)財務コーチングの実技指導を行える
+税理士登録済であること【仮】</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>＜事業を前に進める管理者＞
+(1)法人目標の達成に向けたリアリティある計画（予算策定）ができる人
+(2)所外との交渉・契約締結、部門横断的な働きかけができる人
+(3)リーダーシップを発揮して、組織を精鋭集団にできる人</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>(1)労働分配率43%（部下の売上10%計上）
+(2)担当領域の予算を自ら策定し、期中の軌道修正を含めて達成できる
+(3)ゼロから業務を企画して組織化・収益化する力を有している
+(4)6名以上の組織を運営できる【仮】</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>(1)自らの専門以外の分野にも積極的に関与し、法人視点での経営への提案ができる</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>(1)財務コーチングの実技試験を行える
 (2)所内ハンドブックの更新を提案し、実際に更新ができる</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>経営12カ条（稲盛和夫）
-TQ（Time Quest）
-経営者の条件</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="67.5" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>D・SD</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>拠点長
-－ディレクター</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>D1〜SD3</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>2,386〜3,014万円</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>予算策定と拠点経営</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>＜Dへの昇格要件＞
-所内ハンドブック試験（マネージャー用）
+TQ（Time Quest）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="67.5" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>拠点長</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>D1〜D3</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>2,386〜2,637万円</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>マネジャーの育成</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>＜SDへの昇格要件＞
+所内ハンドブック試験（マネージャー用）【要決定】
 半年間に7冊以上の読書（要レポート）
 宣言書＆面接試験
-税理士試験科目合格3科目以上（または同等と代表が認めるもの）</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+税理士試験科目合格3科目以上（または同等と代表が認めるもの）【仮】</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>＜有能な管理者＞
-(1)法人目標の達成に向けたリアリティある計画（予算策定）と、所外との交渉・契約締結、部門横断的な働きかけができる人
-(2)リーダーシップを発揮して、組織を精鋭集団にできる人
-(3)事務所経営に生じる矛盾を受け入れつつもうまく昇華できる人</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>(1)労働分配率43%（部下の売上10%計上※4）
-(2)6名以上の組織（拠点・部門）を運営できる
+(1)部長（M・SM）以下の指導育成ができる人
+(2)働く幸せの実現に向けて、自己利益より部下利益を優先できる人
+(3)事務所経営に生じる矛盾を受け入れつつ、うまく昇華できる人</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>(1)労働分配率43%（部下の売上10%計上）
+(2)6名以上の組織（拠点・部門）を運営できる【仮】
 (3)担当拠点の財務状況を把握し、単月黒字を達成できている
-(4)ゼロから業務を企画して組織化、収益化する力を有している</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>(1)自らの専門以外の分野にも積極的に関与し、法人視点での経営への提案ができる</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
+(4)自らの専門領域において、部長を率いて自らで判断ができる</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>(1)総務・経理の担当者を育成し、業務の属人化を解消できる</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>(1)定期的に部下を昇格させている
 (2)マニュアルの作成・更新指示を行っている
 (3)所内ハンドブックの更新を提案し、実際に更新ができる</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>生き方（稲盛和夫）
 君に成功を贈る
@@ -872,218 +954,282 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="67.5" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>M・SM</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>部長
-－マネージャー</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>M1〜SM3</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>1,633〜2,261万円</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>部下の育成と
-「何とかしてやる」
-の体現</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>＜Mへの昇格要件＞
-所内ハンドブック試験（マネージャー用）
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>部長</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>SM1〜SM3</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>2,009〜2,261万円</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>チーム間の相乗効果</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>＜Dへの昇格要件＞
+所内ハンドブック試験（マネージャー用）【要決定】
+半年間に6冊以上の読書（要レポート）
+宣言書＆面接試験</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>＜チームをつなぐ管理者＞
+(1)自チームの成果だけでなく、他チームと連携して法人全体の成果を上げられる人
+(2)部門をまたぐ課題を自ら拾い、関係者を巻き込んで解決できる人
+(3)自チームの利益より法人全体の利益を優先できる人</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>(1)労働分配率43%（部下の売上10%計上）
+(2)他チームとの共同案件を主導し、収益化できている
+(3)繁忙期の応援・引き継ぎをチーム間で設計し、特定の個人に負荷が偏らない状態を作れる
+(4)複数チーム（計6名以上）に影響を及ぼす立場にある【仮】</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>(1)部門をまたぐ業務フローの再設計を提案し、実行できる</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>(1)他チームの部長と定例で情報連携している
+(2)チーム間の異動・応援の調整を自ら行っている
+(3)所内ハンドブックの更新を提案し、実際に更新ができる</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>考える技術・書く技術
+絆徳経営のすゝめ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="67.5" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>部長</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>M1〜M3</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>1,633〜1,884万円</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>チーム力の向上</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>＜SMへの昇格要件＞
+所内ハンドブック試験（マネージャー用）【要決定】
 半年間に6冊以上の読書（要レポート）
 宣言書＆面接試験
-財務コーチング養成動画B判定以上</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+財務コーチング養成動画 B判定以上</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>＜チームを持つ管理者＞
-(1)経験ある分野の目標を定め（部下の目標設定を含めて）何とかして達成できる人
-(2)達成に向けた課題や問題を解決する人
+(1)経験ある分野の目標を定め（部下の目標設定を含めて）、何とかして達成できる人
+(2)達成に向けた課題や問題を自ら解決する人
 (3)家族的なチームを作れる人
-(4)主任以下の指導育成ができる人</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>(1)労働分配率43%（部下の売上10%計上※4）
-(2)3名以上の組織を運営できる
-(3)担当関与先の月次巡回監査・決算申告を、期限管理を含めチームで完結できる</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
+(4)主任（SS）以下の指導育成ができる人</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>(1)労働分配率43%（部下の売上10%計上）
+(2)3名以上の組織を運営できる【仮】
+(3)チームの担当関与先の月次巡回監査・決算申告を、期限管理を含めチームで完結できる
+(4)部下一人ひとりの担当先と負荷を把握し、期中で組み替えられる</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>(1)自らの専門領域（税務・労務・システム等）を継続的に追及し、所内の相談窓口になれる</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>(1)所内ハンドブックの更新を提案し、実際に更新ができる
-(2)部下の半期目標の設定・振り返りを実施している</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>EQこころの知能指数
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>(1)部下の半期目標の設定・振り返りを実施している
+(2)所内ハンドブックの更新を提案し、実際に更新ができる</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>EQ こころの知能指数
 レバレッジ時間術
 7つの習慣
 はじめての課長の教科書</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="81" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="9" ht="81" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>SS</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>主任
-－シニアスタッフ</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>主任</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>SS1〜SS6</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>1,193〜1,507万円</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>精鋭集団化への貢献と
-実行の徹底</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>＜SSへの昇格要件＞
-所内ハンドブック試験（スタッフ用）
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>どれだけ自走できるか</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>＜Mへの昇格要件＞
+所内ハンドブック試験（スタッフ用）【要決定】
 半年間に5冊以上の読書（要レポート）
 宣言書＆面接試験
-財務コーチング養成動画C判定以上
-日商簿記2級以上（または税理士試験科目合格1科目以上）</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>＜組織に寄与する個人＞
-(1)（Sの要件に加え、）言われたことの実行徹底ができ、自分の目標を達成できる人
+財務コーチング養成動画 C判定以上
+日商簿記2級以上（または税理士試験科目合格1科目以上）【仮】</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>＜自分で回し切る個人＞
+(1)指示を待たずに自分の担当を回し切り、判断に迷う点だけを上司に上げられる人
 (2)失敗をフィードバックと捉え、挑戦できる人
 (3)質の良い提案書を作成し、周りの人を説得するプランを立案したことがある人</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>(1)労働分配率43%（※4）
-(2)業務マニュアルを使って後輩の指導ができる
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>(1)労働分配率43%
+(2)決算・申告を単独で完結し、関与先へ説明できる
 (3)トレーナーとして担当職（S）を指導できる
-(4)決算・申告を単独で完結し、関与先へ説明できる</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
+(4)担当先からの一次照会を、上司を介さず自ら回答できる</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>(1)所内環境の改善に向けた提案ができる
 (2)業務マニュアルを使って後輩の指導ができる</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>(1)マニュアルを常に更新している（新しい業務は1から作成している）
 (2)半期目標を常に意識して行動している
 (3)自身の時間毎の売上高（生産性）を意識して行動している</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>ストレスフリーの整理術
 絶妙な「報・連・相」の技術
 働き方（稲盛和夫）
-あたりまえだけどなかなかできない仕事のルール
-考える技術・書く技術</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="67.5" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+あたりまえだけどなかなかできない仕事のルール</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="67.5" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>担当職
-－スタッフ</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>担当職</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>S1〜S6</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>816〜1,130万円</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
-        <is>
-          <t>実行の徹底</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>＜Sへの昇格要件＞
-所内ハンドブック試験（スタッフ用）
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>実行力の習得</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>＜SSへの昇格要件＞
+所内ハンドブック試験（スタッフ用）【要決定】
 半年間に5冊以上の読書（要レポート）
 宣言書＆面接試験
-日商簿記3級以上</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
+日商簿記3級以上【仮】</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>＜組織のメンバー＞
 (1)報・連・相を適正に行い、ボールをなるべく持たず、肩から当たりにいける人
 (2)上司からの指示を実行徹底できる人</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>(1)労働分配率43%（※4）
-(2)月次巡回監査を担当先について自ら実施し、期限内に完了できる</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>(1)労働分配率43%
+(2)月次巡回監査を担当先について自ら実施し、期限内に完了できる
+(3)教わった手順を、次からは自分だけで再現できる</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>(1)定型業務を期限内に、指示なく完了できる</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>(1)上司の指示内容を記録し、完了報告まで自分で完結している
 (2)業務マニュアルに沿って作業し、気づいた点を上司に報告している</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>敬語の使い方が面白いほど身につく本
 入社1年目の教科書
@@ -1092,173 +1238,174 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+    <row r="11" ht="67.5" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>研究生
-－アソシエイト</t>
-        </is>
-      </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>研究生</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>754万円</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>基礎の習得</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>＜T1への昇格要件（本採用）＞
-面接
-税理士法人福田会計の理念への共感
-所内ハンドブックの通読</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
+        <is>
+          <t>文化に慣れる</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>＜Sへの昇格要件＞
+所内ハンドブック試験（スタッフ用）【要決定】
+半年間に5冊以上の読書（要レポート）
+宣言書＆面接試験
+日商簿記3級以上【仮】</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>＜これから戦力になる人＞
-(1)教わったことを素直に実行し、同じ指摘を繰り返さない人
-(2)分からないことを、分からないまま放置しない人</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
+(1)理念と所内のやり方に馴染み、教わったことを素直に実行できる人
+(2)同じ指摘を繰り返さない人
+(3)分からないことを、分からないまま放置しない人</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>(1)期待売上高・労働分配率は問わない（賞与は在籍月数按分）
 (2)担当補助として、指示された作業を期限内に完了できる</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>(1)所内ルール（勤怠・報告・ファイル保存）を守れる</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>(1)日報・週報で進捗と不明点を必ず報告している</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>所内ハンドブック
 税理士を活用して業績を3倍にする方法</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
+    <row r="12" ht="52" customHeight="1">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>―</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>入社前</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>試用期間</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr">
         <is>
           <t>―</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>―</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E12" s="23" t="inlineStr">
         <is>
           <t>スムーズな合流</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>＜試用期間修了要件＞
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>＜T1への昇格要件＞
 面接
 税理士法人福田会計の理念（MVV）への共感</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr"/>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr"/>
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr"/>
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>所内ハンドブック
 税理士を活用して業績を3倍にする方法</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="14" customHeight="1">
-      <c r="A12" s="20" t="inlineStr">
+    <row r="14" ht="14" customHeight="1">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>※0.測定指標1は関与先を担当する職員（フロントオフィス）、測定指標2は総務・経理（バックオフィス）に適用する。兼任者は両方を見る。</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="14" customHeight="1">
-      <c r="A13" s="20" t="inlineStr">
+    <row r="15" ht="14" customHeight="1">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>※1.所内ハンドブック試験は半年に1回は受験（再受験）すること。</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="14" customHeight="1">
-      <c r="A14" s="20" t="inlineStr">
-        <is>
-          <t>※2.宣言書：自身が期待職能、パフォーマンスを満たしていることを根拠と共に記した文書。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="14" customHeight="1">
-      <c r="A15" s="20" t="inlineStr">
+    <row r="16" ht="14" customHeight="1">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>※2.宣言書：自身が期待される役割・測定指標を満たしていることを根拠と共に記した文書。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="14" customHeight="1">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>※3.読書は、レポートの提出に伴い、レポート1通ごとに2,000円の補助を支給します。</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>※4.半年間の粗利と自分の給与を比較して、労働分配率を計算。新卒の給与は12ヶ月、中途採用の給与は6ヶ月分は労働分配率の計算上考慮しない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="14" customHeight="1">
-      <c r="A17" s="20" t="inlineStr">
+    <row r="18" ht="14" customHeight="1">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>※4.労働分配率は、半年間の粗利と自分の給与を比較して計算。新卒の給与は12ヶ月、中途採用の給与は6ヶ月分は計算上考慮しない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="14" customHeight="1">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>※5.期待売上高＝基本給上限×2×1.3×1.15×14（千円未満切上）。「グレード制度 基本給テーブル」と一致。</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="14" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
+    <row r="20" ht="14" customHeight="1">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>※6.月平均残業30時間超の場合、評価グレードを引き下げる（S：2グレードダウン／SS〜SM：1グレードダウン／T1：考慮しない）。</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="14" customHeight="1">
-      <c r="A19" s="20" t="inlineStr">
-        <is>
-          <t>※7.タイトルが上がれば上がるほど、抽象度が高まりよく分からないことも多くなります。逆に言うと「意味が分かる人しか、その役職にはなれない」とも言えますね。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="14" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
+    <row r="21" ht="14" customHeight="1">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>※7.職階が上がれば上がるほど、抽象度が高まりよく分からないことも多くなります。逆に言うと「意味が分かる人しか、その職階にはなれない」とも言えますね。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="14" customHeight="1">
+      <c r="A22" s="24" t="inlineStr">
         <is>
           <t>※8.評価面談では、この表の文言そのものを使ってフィードバックする。文言は直属上司が起案し、代表が承認、上司から本人へ通知する。</t>
         </is>
@@ -1266,13 +1413,13 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A22:K22"/>
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A21:K21"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A19:K19"/>
-    <mergeCell ref="A13:K13"/>
     <mergeCell ref="A14:K14"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A17:K17"/>

</xml_diff>

<commit_message>
Set required inputs for T1/S/M and use 虎の巻 as the handbook name
</commit_message>
<xml_diff>
--- a/role-expectations/期待職能_福田会計.xlsx
+++ b/role-expectations/期待職能_福田会計.xlsx
@@ -734,7 +734,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>(1)所内ハンドブック・報酬制度の改定を主導できる
+          <t>(1)虎の巻・報酬制度の改定を主導できる
 (2)後継者育成計画を持ち、実行している</t>
         </is>
       </c>
@@ -774,7 +774,7 @@
       <c r="F4" s="5" t="inlineStr">
         <is>
           <t>＜EPへの昇格要件＞
-所内ハンドブック試験（マネージャー用）【要決定】
+虎の巻試験（マネージャー用）【要決定】
 半年間に10冊以上の読書（要レポート）
 宣言書＆面接試験
 税理士登録済であること【仮】</t>
@@ -804,7 +804,7 @@
       <c r="J4" s="5" t="inlineStr">
         <is>
           <t>(1)財務コーチングの実技指導を行える
-(2)所内ハンドブックの更新を提案し、実際に更新ができる</t>
+(2)虎の巻の更新を提案し、実際に更新ができる</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -843,7 +843,7 @@
       <c r="F5" s="5" t="inlineStr">
         <is>
           <t>＜Pへの昇格要件＞
-所内ハンドブック試験（マネージャー用）【要決定】
+虎の巻試験（マネージャー用）【要決定】
 半年間に8冊以上の読書（要レポート）
 宣言書＆面接試験
 税理士登録済であること【仮】</t>
@@ -873,7 +873,7 @@
       <c r="J5" s="5" t="inlineStr">
         <is>
           <t>(1)財務コーチングの実技試験を行える
-(2)所内ハンドブックの更新を提案し、実際に更新ができる</t>
+(2)虎の巻の更新を提案し、実際に更新ができる</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -912,7 +912,7 @@
       <c r="F6" s="5" t="inlineStr">
         <is>
           <t>＜SDへの昇格要件＞
-所内ハンドブック試験（マネージャー用）【要決定】
+虎の巻試験（マネージャー用）【要決定】
 半年間に7冊以上の読書（要レポート）
 宣言書＆面接試験
 税理士試験科目合格3科目以上（または同等と代表が認めるもの）【仮】</t>
@@ -943,7 +943,7 @@
         <is>
           <t>(1)定期的に部下を昇格させている
 (2)マニュアルの作成・更新指示を行っている
-(3)所内ハンドブックの更新を提案し、実際に更新ができる</t>
+(3)虎の巻の更新を提案し、実際に更新ができる</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -983,7 +983,7 @@
       <c r="F7" s="5" t="inlineStr">
         <is>
           <t>＜Dへの昇格要件＞
-所内ハンドブック試験（マネージャー用）【要決定】
+虎の巻試験（マネージャー用）【要決定】
 半年間に6冊以上の読書（要レポート）
 宣言書＆面接試験</t>
         </is>
@@ -1013,7 +1013,7 @@
         <is>
           <t>(1)他チームの部長と定例で情報連携している
 (2)チーム間の異動・応援の調整を自ら行っている
-(3)所内ハンドブックの更新を提案し、実際に更新ができる</t>
+(3)虎の巻の更新を提案し、実際に更新ができる</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1052,7 +1052,7 @@
       <c r="F8" s="5" t="inlineStr">
         <is>
           <t>＜SMへの昇格要件＞
-所内ハンドブック試験（マネージャー用）【要決定】
+虎の巻試験（マネージャー用）【要決定】
 半年間に6冊以上の読書（要レポート）
 宣言書＆面接試験
 財務コーチング養成動画 B判定以上</t>
@@ -1083,15 +1083,12 @@
       <c r="J8" s="5" t="inlineStr">
         <is>
           <t>(1)部下の半期目標の設定・振り返りを実施している
-(2)所内ハンドブックの更新を提案し、実際に更新ができる</t>
+(2)虎の巻の更新を提案し、実際に更新ができる</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>EQ こころの知能指数
-レバレッジ時間術
-7つの習慣
-はじめての課長の教科書</t>
+          <t>ATC受講</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1121,7 @@
       <c r="F9" s="5" t="inlineStr">
         <is>
           <t>＜Mへの昇格要件＞
-所内ハンドブック試験（スタッフ用）【要決定】
+虎の巻試験（スタッフ用）【要決定】
 半年間に5冊以上の読書（要レポート）
 宣言書＆面接試験
 財務コーチング養成動画 C判定以上
@@ -1162,8 +1159,7 @@
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>ストレスフリーの整理術
-絶妙な「報・連・相」の技術
+          <t>絶妙な「報・連・相」の技術
 働き方（稲盛和夫）
 あたりまえだけどなかなかできない仕事のルール</t>
         </is>
@@ -1198,7 +1194,7 @@
       <c r="F10" s="5" t="inlineStr">
         <is>
           <t>＜SSへの昇格要件＞
-所内ハンドブック試験（スタッフ用）【要決定】
+虎の巻試験（スタッフ用）【要決定】
 半年間に5冊以上の読書（要レポート）
 宣言書＆面接試験
 日商簿記3級以上【仮】</t>
@@ -1231,10 +1227,7 @@
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>敬語の使い方が面白いほど身につく本
-入社1年目の教科書
-伸びる新人は「これ」をやらない!
-脱★ドンブリ経営</t>
+          <t>ロジカルコミュニケーション</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1260,7 @@
       <c r="F11" s="5" t="inlineStr">
         <is>
           <t>＜Sへの昇格要件＞
-所内ハンドブック試験（スタッフ用）【要決定】
+虎の巻試験（スタッフ用）【要決定】
 半年間に5冊以上の読書（要レポート）
 宣言書＆面接試験
 日商簿記3級以上【仮】</t>
@@ -1299,8 +1292,8 @@
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>所内ハンドブック
-税理士を活用して業績を3倍にする方法</t>
+          <t>福田会計虎の巻
+ストレスフリーの仕事術</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1336,7 @@
       <c r="J12" s="5" t="inlineStr"/>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>所内ハンドブック
+          <t>福田会計虎の巻
 税理士を活用して業績を3倍にする方法</t>
         </is>
       </c>
@@ -1358,7 +1351,7 @@
     <row r="15" ht="14" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>※1.所内ハンドブック試験は半年に1回は受験（再受験）すること。</t>
+          <t>※1.虎の巻試験は半年に1回は受験（再受験）すること。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove the 入社前 level; T1 is now the entry point
</commit_message>
<xml_diff>
--- a/role-expectations/期待職能_福田会計.xlsx
+++ b/role-expectations/期待職能_福田会計.xlsx
@@ -69,7 +69,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -126,11 +126,6 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -158,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -221,12 +216,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -597,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1297,108 +1286,64 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="52" customHeight="1">
-      <c r="A12" s="22" t="inlineStr">
-        <is>
-          <t>―</t>
-        </is>
-      </c>
-      <c r="B12" s="22" t="inlineStr">
-        <is>
-          <t>入社前</t>
-        </is>
-      </c>
-      <c r="C12" s="23" t="inlineStr">
-        <is>
-          <t>試用期間</t>
-        </is>
-      </c>
-      <c r="D12" s="23" t="inlineStr">
-        <is>
-          <t>―</t>
-        </is>
-      </c>
-      <c r="E12" s="23" t="inlineStr">
-        <is>
-          <t>スムーズな合流</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>＜T1への昇格要件＞
-面接
-税理士法人福田会計の理念（MVV）への共感</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr"/>
-      <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr"/>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>福田会計虎の巻
-税理士を活用して業績を3倍にする方法</t>
+    <row r="13" ht="14" customHeight="1">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>※0.測定指標1は関与先を担当する職員（フロントオフィス）、測定指標2は総務・経理（バックオフィス）に適用する。兼任者は両方を見る。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>※0.測定指標1は関与先を担当する職員（フロントオフィス）、測定指標2は総務・経理（バックオフィス）に適用する。兼任者は両方を見る。</t>
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>※1.虎の巻試験は半年に1回は受験（再受験）すること。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="14" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>※1.虎の巻試験は半年に1回は受験（再受験）すること。</t>
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>※2.宣言書：自身が期待される役割・測定指標を満たしていることを根拠と共に記した文書。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>※2.宣言書：自身が期待される役割・測定指標を満たしていることを根拠と共に記した文書。</t>
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>※3.読書は、レポートの提出に伴い、レポート1通ごとに2,000円の補助を支給します。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
-        <is>
-          <t>※3.読書は、レポートの提出に伴い、レポート1通ごとに2,000円の補助を支給します。</t>
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>※4.労働分配率は、半年間の粗利と自分の給与を比較して計算。新卒の給与は12ヶ月、中途採用の給与は6ヶ月分は計算上考慮しない。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
-      <c r="A18" s="24" t="inlineStr">
-        <is>
-          <t>※4.労働分配率は、半年間の粗利と自分の給与を比較して計算。新卒の給与は12ヶ月、中途採用の給与は6ヶ月分は計算上考慮しない。</t>
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>※5.期待売上高＝基本給上限×2×1.3×1.15×14（千円未満切上）。「グレード制度 基本給テーブル」と一致。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="14" customHeight="1">
-      <c r="A19" s="24" t="inlineStr">
-        <is>
-          <t>※5.期待売上高＝基本給上限×2×1.3×1.15×14（千円未満切上）。「グレード制度 基本給テーブル」と一致。</t>
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>※6.月平均残業30時間超の場合、評価グレードを引き下げる（S：2グレードダウン／SS〜SM：1グレードダウン／T1：考慮しない）。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="14" customHeight="1">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>※6.月平均残業30時間超の場合、評価グレードを引き下げる（S：2グレードダウン／SS〜SM：1グレードダウン／T1：考慮しない）。</t>
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>※7.職階が上がれば上がるほど、抽象度が高まりよく分からないことも多くなります。逆に言うと「意味が分かる人しか、その職階にはなれない」とも言えますね。</t>
         </is>
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
-      <c r="A21" s="24" t="inlineStr">
-        <is>
-          <t>※7.職階が上がれば上がるほど、抽象度が高まりよく分からないことも多くなります。逆に言うと「意味が分かる人しか、その職階にはなれない」とも言えますね。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="14" customHeight="1">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>※8.評価面談では、この表の文言そのものを使ってフィードバックする。文言は直属上司が起案し、代表が承認、上司から本人へ通知する。</t>
         </is>
@@ -1406,13 +1351,13 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A22:K22"/>
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A20:K20"/>
     <mergeCell ref="A21:K21"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A13:K13"/>
     <mergeCell ref="A14:K14"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A17:K17"/>

</xml_diff>

<commit_message>
Use T as the 研究生 symbol and mark T/S sections provisional
</commit_message>
<xml_diff>
--- a/role-expectations/期待職能_福田会計.xlsx
+++ b/role-expectations/期待職能_福田会計.xlsx
@@ -1154,7 +1154,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="67.5" customHeight="1">
+    <row r="10" ht="81" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>S</t>
@@ -1182,7 +1182,8 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>＜SSへの昇格要件＞
+          <t>【仮】
+＜SSへの昇格要件＞
 虎の巻試験（スタッフ用）【要決定】
 半年間に5冊以上の読書（要レポート）
 宣言書＆面接試験
@@ -1191,14 +1192,16 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>＜組織のメンバー＞
+          <t>【仮】
+＜組織のメンバー＞
 (1)報・連・相を適正に行い、ボールをなるべく持たず、肩から当たりにいける人
 (2)上司からの指示を実行徹底できる人</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>(1)労働分配率43%
+          <t>【仮】
+(1)労働分配率43%
 (2)月次巡回監査を担当先について自ら実施し、期限内に完了できる
 (3)教わった手順を、次からは自分だけで再現できる</t>
         </is>
@@ -1220,22 +1223,22 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="67.5" customHeight="1">
+    <row r="11" ht="81" customHeight="1">
       <c r="A11" s="20" t="inlineStr">
         <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>研究生</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>研究生</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
           <t>754万円</t>
@@ -1248,7 +1251,8 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>＜Sへの昇格要件＞
+          <t>【仮】
+＜Sへの昇格要件＞
 虎の巻試験（スタッフ用）【要決定】
 半年間に5冊以上の読書（要レポート）
 宣言書＆面接試験
@@ -1331,7 +1335,7 @@
     <row r="19" ht="14" customHeight="1">
       <c r="A19" s="22" t="inlineStr">
         <is>
-          <t>※6.月平均残業30時間超の場合、評価グレードを引き下げる（S：2グレードダウン／SS〜SM：1グレードダウン／T1：考慮しない）。</t>
+          <t>※6.月平均残業30時間超の場合、評価グレードを引き下げる（S：2グレードダウン／SS〜SM：1グレードダウン／T：考慮しない）。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add manual-improvement expectations to T and S roles
</commit_message>
<xml_diff>
--- a/role-expectations/期待職能_福田会計.xlsx
+++ b/role-expectations/期待職能_福田会計.xlsx
@@ -1195,7 +1195,8 @@
           <t>【仮】
 ＜組織のメンバー＞
 (1)報・連・相を適正に行い、ボールをなるべく持たず、肩から当たりにいける人
-(2)上司からの指示を実行徹底できる人</t>
+(2)上司からの指示を実行徹底できる人
+(3)所内マニュアルの誤りや不足に気づき、改善案まで出せる人</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1264,7 +1265,8 @@
           <t>＜これから戦力になる人＞
 (1)理念と所内のやり方に馴染み、教わったことを素直に実行できる人
 (2)同じ指摘を繰り返さない人
-(3)分からないことを、分からないまま放置しない人</t>
+(3)分からないことを、分からないまま放置しない人
+(4)所内マニュアルの分かりにくい箇所・古い箇所に気づき、上司に伝えられる人</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Move T/S manual-improvement items from role to 測定指標2
</commit_message>
<xml_diff>
--- a/role-expectations/期待職能_福田会計.xlsx
+++ b/role-expectations/期待職能_福田会計.xlsx
@@ -1195,8 +1195,7 @@
           <t>【仮】
 ＜組織のメンバー＞
 (1)報・連・相を適正に行い、ボールをなるべく持たず、肩から当たりにいける人
-(2)上司からの指示を実行徹底できる人
-(3)所内マニュアルの誤りや不足に気づき、改善案まで出せる人</t>
+(2)上司からの指示を実行徹底できる人</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1209,7 +1208,8 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>(1)定型業務を期限内に、指示なく完了できる</t>
+          <t>(1)定型業務を期限内に、指示なく完了できる
+(2)所内マニュアルの誤りや不足に気づき、改善案まで出せている</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1265,8 +1265,7 @@
           <t>＜これから戦力になる人＞
 (1)理念と所内のやり方に馴染み、教わったことを素直に実行できる人
 (2)同じ指摘を繰り返さない人
-(3)分からないことを、分からないまま放置しない人
-(4)所内マニュアルの分かりにくい箇所・古い箇所に気づき、上司に伝えられる人</t>
+(3)分からないことを、分からないまま放置しない人</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1277,7 +1276,8 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>(1)所内ルール（勤怠・報告・ファイル保存）を守れる</t>
+          <t>(1)所内ルール（勤怠・報告・ファイル保存）を守れる
+(2)所内マニュアルの分かりにくい箇所・古い箇所に気づき、上司に伝えている</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">

</xml_diff>